<commit_message>
Decks: add section 00 (ns-3/VMware setup, first 4-node experiment) at start, related-mechanisms and references slides; add refs 10-15 to report and workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019rZdtfEbJpAbmcB9G79J6K
</commit_message>
<xml_diff>
--- a/thesis-final/WSN_Protocol_Comparison.xlsx
+++ b/thesis-final/WSN_Protocol_Comparison.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="262">
   <si>
     <t xml:space="preserve">WSN Clustering Protocols — Comparison Workbook</t>
   </si>
@@ -254,6 +254,42 @@
   </si>
   <si>
     <t xml:space="preserve">El-Sayed, Abd-Elgaber and Refaay, “An Intelligent RL Enhanced Improved LEACH Protocol for Prolonging WSN Lifetime,” Scientific Reports, 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[10]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J. Jassbi and S. Moridi, “Fault Tolerance and Energy Efficient Clustering Algorithm in Wireless Sensor Networks: FTEC,” Wireless Personal Communications, 2019. doi:10.1007/s11277-019-06281-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[11]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R. Pachlor, D. Shrimankar, K. K. Nagwanshi and M. Paliwal, “Cluster-Head Rotation Approaches in Sensor Networks: A Review,” arXiv:2206.08892, 2022.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[12]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. Li, M. Ye, G. Chen and J. Wu, “An Energy-Efficient Unequal Clustering Mechanism for Wireless Sensor Networks,” Proc. IEEE MASS, 2005.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[13]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V. Chauhan and S. Soni, “Energy Aware Unequal Clustering Algorithm with Multi-hop Routing via Low Degree Relay Nodes for Wireless Sensor Networks,” J. Ambient Intelligence and Humanized Computing, vol. 12, pp. 2469–2482, 2021. doi:10.1007/s12652-020-02385-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[14]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W. B. Heinzelman, A. P. Chandrakasan and H. Balakrishnan, “An Application-Specific Protocol Architecture for Wireless Microsensor Networks,” IEEE Trans. Wireless Communications, 2002.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[15]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ns-3 Network Simulator, release 3.41, https://www.nsnam.org</t>
   </si>
   <si>
     <t xml:space="preserve">Dashboard — best configuration of each family (BS center)</t>
@@ -1670,11 +1706,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="27347994"/>
-        <c:axId val="84565287"/>
+        <c:axId val="8582350"/>
+        <c:axId val="66080545"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="27347994"/>
+        <c:axId val="8582350"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1706,7 +1742,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84565287"/>
+        <c:crossAx val="66080545"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1714,7 +1750,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="84565287"/>
+        <c:axId val="66080545"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1756,7 +1792,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27347994"/>
+        <c:crossAx val="8582350"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1980,11 +2016,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="94471764"/>
-        <c:axId val="91881181"/>
+        <c:axId val="92750844"/>
+        <c:axId val="69968752"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="94471764"/>
+        <c:axId val="92750844"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2016,7 +2052,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91881181"/>
+        <c:crossAx val="69968752"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2024,7 +2060,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="91881181"/>
+        <c:axId val="69968752"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2068,7 +2104,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94471764"/>
+        <c:crossAx val="92750844"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2616,11 +2652,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="44673727"/>
-        <c:axId val="9308125"/>
+        <c:axId val="62941431"/>
+        <c:axId val="19910775"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="44673727"/>
+        <c:axId val="62941431"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2652,7 +2688,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9308125"/>
+        <c:crossAx val="19910775"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2660,7 +2696,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9308125"/>
+        <c:axId val="19910775"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2736,7 +2772,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44673727"/>
+        <c:crossAx val="62941431"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3129,11 +3165,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="72231332"/>
-        <c:axId val="11218485"/>
+        <c:axId val="91499267"/>
+        <c:axId val="99570618"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="72231332"/>
+        <c:axId val="91499267"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3165,7 +3201,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11218485"/>
+        <c:crossAx val="99570618"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3173,7 +3209,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11218485"/>
+        <c:axId val="99570618"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3249,7 +3285,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72231332"/>
+        <c:crossAx val="91499267"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3311,8 +3347,8 @@
       <xdr:rowOff>131040</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>331200</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>354960</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>113040</xdr:rowOff>
     </xdr:to>
@@ -3322,7 +3358,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7959600" y="571680"/>
+        <a:off x="7168680" y="571680"/>
         <a:ext cx="7919640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -3341,8 +3377,8 @@
       <xdr:rowOff>131040</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>331200</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>354960</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>163440</xdr:rowOff>
     </xdr:to>
@@ -3352,7 +3388,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="7959600" y="4400640"/>
+        <a:off x="7168680" y="4400640"/>
         <a:ext cx="7919640" cy="2699640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -3376,8 +3412,8 @@
       <xdr:rowOff>130680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>3600</xdr:colOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>160560</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>131760</xdr:rowOff>
     </xdr:to>
@@ -3387,7 +3423,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="9867960" y="4971960"/>
+        <a:off x="8881200" y="4971960"/>
         <a:ext cx="8639640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -3412,7 +3448,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>87480</xdr:colOff>
+      <xdr:colOff>798840</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>142560</xdr:rowOff>
     </xdr:to>
@@ -3616,8 +3652,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B51"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
@@ -3870,7 +3906,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
         <v>58</v>
       </c>
@@ -3878,7 +3914,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
         <v>60</v>
       </c>
@@ -3926,7 +3962,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
         <v>72</v>
       </c>
@@ -3940,6 +3976,54 @@
       </c>
       <c r="B45" s="5" t="s">
         <v>75</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -3959,7 +4043,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F19"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
@@ -3968,29 +4052,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>24</v>
@@ -3998,10 +4082,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A5)*('Unified Comparison'!$C$5:$C$28=B5),0),0))</f>
@@ -4022,10 +4106,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A6)*('Unified Comparison'!$C$5:$C$28=B6),0),0))</f>
@@ -4046,10 +4130,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A7)*('Unified Comparison'!$C$5:$C$28=B7),0),0))</f>
@@ -4070,10 +4154,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A8)*('Unified Comparison'!$C$5:$C$28=B8),0),0))</f>
@@ -4094,10 +4178,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="C9" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A9)*('Unified Comparison'!$C$5:$C$28=B9),0),0))</f>
@@ -4118,10 +4202,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A10)*('Unified Comparison'!$C$5:$C$28=B10),0),0))</f>
@@ -4142,10 +4226,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="C11" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A11)*('Unified Comparison'!$C$5:$C$28=B11),0),0))</f>
@@ -4166,10 +4250,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="C12" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A12)*('Unified Comparison'!$C$5:$C$28=B12),0),0))</f>
@@ -4190,10 +4274,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="C13" s="12" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A13)*('Unified Comparison'!$C$5:$C$28=B13),0),0))</f>
@@ -4214,12 +4298,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="C16" s="15" t="n">
         <f aca="false">C13/C9-1</f>
@@ -4228,7 +4312,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="C17" s="15" t="n">
         <f aca="false">C13/C5-1</f>
@@ -4237,7 +4321,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="C18" s="16" t="n">
         <f aca="false">(F13-F11)*100</f>
@@ -4246,7 +4330,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="C19" s="15" t="n">
         <f aca="false">'Center vs Far BS'!F9/'Center vs Far BS'!F7-1</f>
@@ -4271,7 +4355,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:L30"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
@@ -4285,64 +4369,64 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>24</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>1409</v>
@@ -4375,16 +4459,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="E6" s="24" t="n">
         <v>323</v>
@@ -4417,16 +4501,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>338</v>
@@ -4459,16 +4543,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="E8" s="24" t="n">
         <v>1324</v>
@@ -4501,16 +4585,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>1440</v>
@@ -4543,16 +4627,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="E10" s="24" t="n">
         <v>1247</v>
@@ -4585,16 +4669,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E11" s="18" t="n">
         <v>2177</v>
@@ -4627,16 +4711,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="E12" s="24" t="n">
         <v>2347</v>
@@ -4669,16 +4753,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>1653</v>
@@ -4711,16 +4795,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="E14" s="24" t="n">
         <v>2502</v>
@@ -4753,16 +4837,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="E15" s="18" t="n">
         <v>330</v>
@@ -4795,16 +4879,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E16" s="24" t="n">
         <v>345</v>
@@ -4837,16 +4921,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E17" s="18" t="n">
         <v>1730</v>
@@ -4879,16 +4963,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="E18" s="24" t="n">
         <v>1513</v>
@@ -4921,16 +5005,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="E19" s="18" t="n">
         <v>1513</v>
@@ -4963,16 +5047,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="E20" s="24" t="n">
         <v>1730</v>
@@ -5005,16 +5089,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="E21" s="18" t="n">
         <v>1621</v>
@@ -5047,16 +5131,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="E22" s="24" t="n">
         <v>1551</v>
@@ -5089,16 +5173,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="E23" s="18" t="n">
         <v>1551</v>
@@ -5131,16 +5215,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B24" s="22" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="E24" s="24" t="n">
         <v>1491</v>
@@ -5173,16 +5257,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="E25" s="18" t="n">
         <v>1381</v>
@@ -5215,16 +5299,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="E26" s="24" t="n">
         <v>1730</v>
@@ -5257,16 +5341,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="29" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B27" s="29" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="E27" s="31" t="n">
         <v>2621</v>
@@ -5299,16 +5383,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="29" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B28" s="29" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="E28" s="31" t="n">
         <v>2621</v>
@@ -5341,7 +5425,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="35" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -5361,7 +5445,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:O12"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="11"/>
@@ -5373,64 +5457,64 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>932</v>
@@ -5471,21 +5555,21 @@
         <v>0.485238455715367</v>
       </c>
       <c r="N5" s="28" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="O5" s="28" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="D6" s="24" t="n">
         <v>1106</v>
@@ -5520,15 +5604,15 @@
         <v>-0.317635270541082</v>
       </c>
       <c r="N6" s="23" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="O6" s="23" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>1578</v>
@@ -5569,21 +5653,21 @@
         <v>0.332256575911398</v>
       </c>
       <c r="N7" s="28" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="O7" s="28" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="D8" s="24" t="n">
         <v>493</v>
@@ -5618,18 +5702,18 @@
         <v>0.81447963800905</v>
       </c>
       <c r="N8" s="22" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="O8" s="23" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="C9" s="18" t="n">
         <v>4312</v>
@@ -5667,15 +5751,15 @@
         <v>0.90495867768595</v>
       </c>
       <c r="N9" s="28" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="O9" s="28" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="B10" s="24" t="n">
         <v>1250</v>
@@ -5716,15 +5800,15 @@
         <v>0.934455270150576</v>
       </c>
       <c r="N10" s="22" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="O10" s="23" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="35" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -5744,7 +5828,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:L41"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
@@ -5757,64 +5841,64 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>24</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="E5" s="18" t="n">
         <v>330</v>
@@ -5829,13 +5913,13 @@
         <v>0.9974</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="J5" s="20" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="K5" s="38" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="L5" s="20" t="n">
         <f aca="false">G5/$G$5-1</f>
@@ -5844,16 +5928,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C6" s="22" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E6" s="24" t="n">
         <v>345</v>
@@ -5886,16 +5970,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E7" s="18" t="n">
         <v>1730</v>
@@ -5928,16 +6012,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C8" s="22" t="n">
         <v>15</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="E8" s="24" t="n">
         <v>1513</v>
@@ -5970,16 +6054,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>15</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>1513</v>
@@ -6012,16 +6096,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C10" s="22" t="n">
         <v>5</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="E10" s="24" t="n">
         <v>1730</v>
@@ -6054,16 +6138,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>10</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="E11" s="18" t="n">
         <v>1621</v>
@@ -6096,16 +6180,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C12" s="22" t="n">
         <v>5</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="E12" s="24" t="n">
         <v>1551</v>
@@ -6138,16 +6222,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>1551</v>
@@ -6180,16 +6264,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C14" s="22" t="n">
         <v>5</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="E14" s="24" t="n">
         <v>1266</v>
@@ -6222,16 +6306,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C15" s="17" t="n">
         <v>5</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="E15" s="18" t="n">
         <v>1266</v>
@@ -6264,16 +6348,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C16" s="22" t="n">
         <v>5</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="E16" s="24" t="n">
         <v>1491</v>
@@ -6306,16 +6390,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C17" s="17" t="n">
         <v>10</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="E17" s="18" t="n">
         <v>1381</v>
@@ -6348,16 +6432,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C18" s="22" t="n">
         <v>5</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="E18" s="24" t="n">
         <v>1730</v>
@@ -6390,16 +6474,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="29" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B19" s="29" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C19" s="29" t="n">
         <v>5</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="E19" s="31" t="n">
         <v>2621</v>
@@ -6432,16 +6516,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="29" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="B20" s="29" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C20" s="29" t="n">
         <v>5</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="E20" s="31" t="n">
         <v>1471</v>
@@ -6474,16 +6558,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="29" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="B21" s="29" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C21" s="29" t="n">
         <v>5</v>
       </c>
       <c r="D21" s="30" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="E21" s="31" t="n">
         <v>2621</v>
@@ -6516,16 +6600,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="29" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="B22" s="29" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C22" s="29" t="n">
         <v>5</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="E22" s="31" t="n">
         <v>1716</v>
@@ -6558,26 +6642,26 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="35" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="41" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="42" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="B27" s="42" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="C27" s="42" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="D27" s="42" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="E27" s="42" t="s">
         <v>24</v>
@@ -6909,7 +6993,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="0" width="10"/>
@@ -6918,55 +7002,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>1730</v>
@@ -7007,7 +7091,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="B6" s="24" t="n">
         <v>1551</v>
@@ -7048,7 +7132,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>1551</v>
@@ -7089,7 +7173,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="B8" s="24" t="n">
         <v>2621</v>
@@ -7130,7 +7214,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="B9" s="31" t="n">
         <v>2621</v>
@@ -7187,7 +7271,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
@@ -7199,54 +7283,54 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="29" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="C6" s="31" t="n">
         <v>2621</v>
@@ -7274,10 +7358,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>2621</v>
@@ -7305,10 +7389,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="C8" s="18" t="n">
         <v>2585</v>
@@ -7336,10 +7420,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>2621</v>
@@ -7367,10 +7451,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="C10" s="18" t="n">
         <v>1821</v>
@@ -7398,10 +7482,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>2171</v>
@@ -7429,10 +7513,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="C12" s="18" t="n">
         <v>1730</v>
@@ -7460,47 +7544,47 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C17" s="18" t="n">
         <v>2621</v>
@@ -7529,10 +7613,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>2566</v>
@@ -7561,10 +7645,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="B19" s="29" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C19" s="31" t="n">
         <v>2621</v>
@@ -7593,10 +7677,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C20" s="24" t="n">
         <v>1471</v>
@@ -7625,10 +7709,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C21" s="18" t="n">
         <v>1696</v>
@@ -7657,10 +7741,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="30" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="B22" s="29" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C22" s="31" t="n">
         <v>1716</v>
@@ -7689,35 +7773,35 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C27" s="18" t="n">
         <v>1688</v>
@@ -7734,10 +7818,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="29" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="B28" s="29" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="C28" s="31" t="n">
         <v>2618</v>
@@ -7754,10 +7838,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C29" s="18" t="n">
         <v>1152</v>
@@ -7774,10 +7858,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="29" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="B30" s="29" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C30" s="31" t="n">
         <v>1487</v>
@@ -7794,7 +7878,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="35" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Propagate paper-fidelity fixes to LEACH/HEED/PEGASIS EDITED codes and update all thesis files
- EDITED codes now share the corrected ORIGINAL algorithms (only the
  environment differs); new heed_fairness_EDITED_unified.cc.
- Unified results: LEACH 1383/1586/1842/99.40%, HEED 634/1216/1883/99.68%,
  HEED (fairness) 743/1154/1960/99.74%, PEGASIS 1324/2352/3504/99.42%.
- Paper-exact: LEACH 1035/1152/1327, HEED (N=500) 734/1384/2259,
  PEGASIS 1616/2017/2186.
- PDR claim reworded: v8-Chain has the highest PDR among protocols whose
  first node survives past round 2000 (not the highest overall).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019rZdtfEbJpAbmcB9G79J6K
</commit_message>
<xml_diff>
--- a/thesis-final/WSN_Protocol_Comparison.xlsx
+++ b/thesis-final/WSN_Protocol_Comparison.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="263">
   <si>
     <t xml:space="preserve">WSN Clustering Protocols — Comparison Workbook</t>
   </si>
@@ -559,22 +559,25 @@
     <t xml:space="preserve">Published source</t>
   </si>
   <si>
+    <t xml:space="preserve">50×50 m, far BS, single-term radio, setup cost not charged (as in paper)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heinzelman et al., 2000 — Table 2 (0.5 J)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">graph only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N = 500, sink (50,175), E0 = 2 J, 125-byte packet, 5 frames/round</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Younis &amp; Fahmy, 2004 — graph only (Fig. 8a/8b)</t>
+  </si>
+  <si>
     <t xml:space="preserve">50×50 m, far BS, single-term radio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heinzelman et al., 2000 — Table 2 (0.5 J)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n/a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">graph only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 2 config, far BS, E0 = 2 J, 800-bit packet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Younis &amp; Fahmy, 2004 — graph only (Fig. 8a/8b)</t>
   </si>
   <si>
     <t xml:space="preserve">Lindsey &amp; Raghavendra, 2002 — Table 1 (50×50 m)</t>
@@ -1430,10 +1433,10 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>1409</c:v>
+                  <c:v>1383</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>323</c:v>
+                  <c:v>634</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1324</c:v>
@@ -1552,13 +1555,13 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>1626</c:v>
+                  <c:v>1586</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>570</c:v>
+                  <c:v>1216</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2353</c:v>
+                  <c:v>2352</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>1600</c:v>
@@ -1674,13 +1677,13 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>1962</c:v>
+                  <c:v>1842</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1362</c:v>
+                  <c:v>1883</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2887</c:v>
+                  <c:v>3504</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>1649</c:v>
@@ -1706,11 +1709,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="8582350"/>
-        <c:axId val="66080545"/>
+        <c:axId val="46280220"/>
+        <c:axId val="52162433"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="8582350"/>
+        <c:axId val="46280220"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1742,7 +1745,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66080545"/>
+        <c:crossAx val="52162433"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1750,7 +1753,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="66080545"/>
+        <c:axId val="52162433"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1792,7 +1795,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8582350"/>
+        <c:crossAx val="46280220"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1984,13 +1987,13 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.9837</c:v>
+                  <c:v>0.994</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.9969</c:v>
+                  <c:v>0.9968</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.9867</c:v>
+                  <c:v>0.9942</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0.9979</c:v>
@@ -2016,11 +2019,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="92750844"/>
-        <c:axId val="69968752"/>
+        <c:axId val="39719945"/>
+        <c:axId val="25492708"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="92750844"/>
+        <c:axId val="39719945"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2052,7 +2055,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69968752"/>
+        <c:crossAx val="25492708"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2060,7 +2063,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69968752"/>
+        <c:axId val="25492708"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2104,7 +2107,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92750844"/>
+        <c:crossAx val="39719945"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2652,11 +2655,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="62941431"/>
-        <c:axId val="19910775"/>
+        <c:axId val="36069653"/>
+        <c:axId val="94008186"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="62941431"/>
+        <c:axId val="36069653"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2688,7 +2691,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19910775"/>
+        <c:crossAx val="94008186"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2696,7 +2699,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19910775"/>
+        <c:axId val="94008186"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2772,7 +2775,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62941431"/>
+        <c:crossAx val="36069653"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3165,11 +3168,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="91499267"/>
-        <c:axId val="99570618"/>
+        <c:axId val="97603401"/>
+        <c:axId val="69793482"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="91499267"/>
+        <c:axId val="97603401"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3201,7 +3204,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99570618"/>
+        <c:crossAx val="69793482"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3209,7 +3212,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="99570618"/>
+        <c:axId val="69793482"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3285,7 +3288,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91499267"/>
+        <c:crossAx val="97603401"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4089,19 +4092,19 @@
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A5)*('Unified Comparison'!$C$5:$C$28=B5),0),0))</f>
-        <v>1409</v>
+        <v>1383</v>
       </c>
       <c r="D5" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$F$5:$F$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A5)*('Unified Comparison'!$C$5:$C$28=B5),0),0))</f>
-        <v>1626</v>
+        <v>1586</v>
       </c>
       <c r="E5" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$G$5:$G$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A5)*('Unified Comparison'!$C$5:$C$28=B5),0),0))</f>
-        <v>1962</v>
+        <v>1842</v>
       </c>
       <c r="F5" s="9" t="n">
         <f aca="false">INDEX('Unified Comparison'!$H$5:$H$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A5)*('Unified Comparison'!$C$5:$C$28=B5),0),0))</f>
-        <v>0.9837</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4113,19 +4116,19 @@
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A6)*('Unified Comparison'!$C$5:$C$28=B6),0),0))</f>
-        <v>323</v>
+        <v>634</v>
       </c>
       <c r="D6" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$F$5:$F$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A6)*('Unified Comparison'!$C$5:$C$28=B6),0),0))</f>
-        <v>570</v>
+        <v>1216</v>
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$G$5:$G$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A6)*('Unified Comparison'!$C$5:$C$28=B6),0),0))</f>
-        <v>1362</v>
+        <v>1883</v>
       </c>
       <c r="F6" s="11" t="n">
         <f aca="false">INDEX('Unified Comparison'!$H$5:$H$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A6)*('Unified Comparison'!$C$5:$C$28=B6),0),0))</f>
-        <v>0.9969</v>
+        <v>0.9968</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4141,15 +4144,15 @@
       </c>
       <c r="D7" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$F$5:$F$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A7)*('Unified Comparison'!$C$5:$C$28=B7),0),0))</f>
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="E7" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$G$5:$G$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A7)*('Unified Comparison'!$C$5:$C$28=B7),0),0))</f>
-        <v>2887</v>
+        <v>3504</v>
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">INDEX('Unified Comparison'!$H$5:$H$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A7)*('Unified Comparison'!$C$5:$C$28=B7),0),0))</f>
-        <v>0.9867</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4316,7 +4319,7 @@
       </c>
       <c r="C17" s="15" t="n">
         <f aca="false">C13/C5-1</f>
-        <v>0.860184528034067</v>
+        <v>0.895155459146782</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4429,16 +4432,16 @@
         <v>122</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>1409</v>
+        <v>1383</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>1626</v>
+        <v>1586</v>
       </c>
       <c r="G5" s="18" t="n">
-        <v>1962</v>
+        <v>1842</v>
       </c>
       <c r="H5" s="19" t="n">
-        <v>0.9837</v>
+        <v>0.994</v>
       </c>
       <c r="I5" s="20" t="n">
         <f aca="false">G5/$G$5-1</f>
@@ -4446,15 +4449,15 @@
       </c>
       <c r="J5" s="21" t="n">
         <f aca="false">E5/G5</f>
-        <v>0.718144750254842</v>
+        <v>0.750814332247557</v>
       </c>
       <c r="K5" s="17" t="n">
         <f aca="false">RANK(G5,$G$5:$G$28)</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L5" s="17" t="n">
         <f aca="false">RANK(H5,$H$5:$H$28)</f>
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4471,32 +4474,32 @@
         <v>123</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>323</v>
+        <v>634</v>
       </c>
       <c r="F6" s="24" t="n">
-        <v>570</v>
+        <v>1216</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>1362</v>
+        <v>1883</v>
       </c>
       <c r="H6" s="25" t="n">
-        <v>0.9969</v>
+        <v>0.9968</v>
       </c>
       <c r="I6" s="26" t="n">
         <f aca="false">G6/$G$5-1</f>
-        <v>-0.305810397553517</v>
+        <v>0.0222584147665581</v>
       </c>
       <c r="J6" s="27" t="n">
         <f aca="false">E6/G6</f>
-        <v>0.237151248164464</v>
+        <v>0.336696760488582</v>
       </c>
       <c r="K6" s="22" t="n">
         <f aca="false">RANK(G6,$G$5:$G$28)</f>
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="L6" s="22" t="n">
         <f aca="false">RANK(H6,$H$5:$H$28)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4513,32 +4516,32 @@
         <v>126</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>338</v>
+        <v>743</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>549</v>
+        <v>1154</v>
       </c>
       <c r="G7" s="18" t="n">
-        <v>1502</v>
+        <v>1960</v>
       </c>
       <c r="H7" s="19" t="n">
-        <v>0.9967</v>
+        <v>0.9974</v>
       </c>
       <c r="I7" s="20" t="n">
         <f aca="false">G7/$G$5-1</f>
-        <v>-0.234454638124363</v>
+        <v>0.0640608034744843</v>
       </c>
       <c r="J7" s="21" t="n">
         <f aca="false">E7/G7</f>
-        <v>0.225033288948069</v>
+        <v>0.379081632653061</v>
       </c>
       <c r="K7" s="17" t="n">
         <f aca="false">RANK(G7,$G$5:$G$28)</f>
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="L7" s="17" t="n">
         <f aca="false">RANK(H7,$H$5:$H$28)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4558,29 +4561,29 @@
         <v>1324</v>
       </c>
       <c r="F8" s="24" t="n">
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>2887</v>
+        <v>3504</v>
       </c>
       <c r="H8" s="25" t="n">
-        <v>0.9867</v>
+        <v>0.9942</v>
       </c>
       <c r="I8" s="26" t="n">
         <f aca="false">G8/$G$5-1</f>
-        <v>0.471457696228338</v>
+        <v>0.90228013029316</v>
       </c>
       <c r="J8" s="27" t="n">
         <f aca="false">E8/G8</f>
-        <v>0.458607551091098</v>
+        <v>0.377853881278539</v>
       </c>
       <c r="K8" s="22" t="n">
         <f aca="false">RANK(G8,$G$5:$G$28)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L8" s="22" t="n">
         <f aca="false">RANK(H8,$H$5:$H$28)</f>
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4610,7 +4613,7 @@
       </c>
       <c r="I9" s="20" t="n">
         <f aca="false">G9/$G$5-1</f>
-        <v>-0.182466870540265</v>
+        <v>-0.129207383279044</v>
       </c>
       <c r="J9" s="21" t="n">
         <f aca="false">E9/G9</f>
@@ -4618,11 +4621,11 @@
       </c>
       <c r="K9" s="17" t="n">
         <f aca="false">RANK(G9,$G$5:$G$28)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="L9" s="17" t="n">
         <f aca="false">RANK(H9,$H$5:$H$28)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4652,7 +4655,7 @@
       </c>
       <c r="I10" s="26" t="n">
         <f aca="false">G10/$G$5-1</f>
-        <v>-0.159531090723751</v>
+        <v>-0.104777415852334</v>
       </c>
       <c r="J10" s="27" t="n">
         <f aca="false">E10/G10</f>
@@ -4660,7 +4663,7 @@
       </c>
       <c r="K10" s="22" t="n">
         <f aca="false">RANK(G10,$G$5:$G$28)</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="L10" s="22" t="n">
         <f aca="false">RANK(H10,$H$5:$H$28)</f>
@@ -4694,7 +4697,7 @@
       </c>
       <c r="I11" s="20" t="n">
         <f aca="false">G11/$G$5-1</f>
-        <v>0.174821610601427</v>
+        <v>0.251357220412595</v>
       </c>
       <c r="J11" s="21" t="n">
         <f aca="false">E11/G11</f>
@@ -4736,7 +4739,7 @@
       </c>
       <c r="I12" s="26" t="n">
         <f aca="false">G12/$G$5-1</f>
-        <v>0.273700305810398</v>
+        <v>0.356677524429967</v>
       </c>
       <c r="J12" s="27" t="n">
         <f aca="false">E12/G12</f>
@@ -4778,7 +4781,7 @@
       </c>
       <c r="I13" s="20" t="n">
         <f aca="false">G13/$G$5-1</f>
-        <v>0.113149847094801</v>
+        <v>0.185667752442997</v>
       </c>
       <c r="J13" s="21" t="n">
         <f aca="false">E13/G13</f>
@@ -4820,7 +4823,7 @@
       </c>
       <c r="I14" s="26" t="n">
         <f aca="false">G14/$G$5-1</f>
-        <v>0.940876656472987</v>
+        <v>1.06731813246471</v>
       </c>
       <c r="J14" s="27" t="n">
         <f aca="false">E14/G14</f>
@@ -4862,7 +4865,7 @@
       </c>
       <c r="I15" s="20" t="n">
         <f aca="false">G15/$G$5-1</f>
-        <v>-0.328236493374108</v>
+        <v>-0.284473398479913</v>
       </c>
       <c r="J15" s="21" t="n">
         <f aca="false">E15/G15</f>
@@ -4904,7 +4907,7 @@
       </c>
       <c r="I16" s="26" t="n">
         <f aca="false">G16/$G$5-1</f>
-        <v>-0.290010193679918</v>
+        <v>-0.243756786102063</v>
       </c>
       <c r="J16" s="27" t="n">
         <f aca="false">E16/G16</f>
@@ -4912,7 +4915,7 @@
       </c>
       <c r="K16" s="22" t="n">
         <f aca="false">RANK(G16,$G$5:$G$28)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L16" s="22" t="n">
         <f aca="false">RANK(H16,$H$5:$H$28)</f>
@@ -4946,7 +4949,7 @@
       </c>
       <c r="I17" s="20" t="n">
         <f aca="false">G17/$G$5-1</f>
-        <v>0.377675840978593</v>
+        <v>0.46742671009772</v>
       </c>
       <c r="J17" s="21" t="n">
         <f aca="false">E17/G17</f>
@@ -4988,7 +4991,7 @@
       </c>
       <c r="I18" s="26" t="n">
         <f aca="false">G18/$G$5-1</f>
-        <v>0.284913353720693</v>
+        <v>0.368621064060803</v>
       </c>
       <c r="J18" s="27" t="n">
         <f aca="false">E18/G18</f>
@@ -5030,7 +5033,7 @@
       </c>
       <c r="I19" s="20" t="n">
         <f aca="false">G19/$G$5-1</f>
-        <v>0.231396534148828</v>
+        <v>0.311617806731813</v>
       </c>
       <c r="J19" s="21" t="n">
         <f aca="false">E19/G19</f>
@@ -5072,7 +5075,7 @@
       </c>
       <c r="I20" s="26" t="n">
         <f aca="false">G20/$G$5-1</f>
-        <v>0.0988786952089704</v>
+        <v>0.170466883821933</v>
       </c>
       <c r="J20" s="27" t="n">
         <f aca="false">E20/G20</f>
@@ -5114,7 +5117,7 @@
       </c>
       <c r="I21" s="20" t="n">
         <f aca="false">G21/$G$5-1</f>
-        <v>0.167686034658512</v>
+        <v>0.243756786102063</v>
       </c>
       <c r="J21" s="21" t="n">
         <f aca="false">E21/G21</f>
@@ -5156,7 +5159,7 @@
       </c>
       <c r="I22" s="26" t="n">
         <f aca="false">G22/$G$5-1</f>
-        <v>0.073394495412844</v>
+        <v>0.143322475570033</v>
       </c>
       <c r="J22" s="27" t="n">
         <f aca="false">E22/G22</f>
@@ -5198,7 +5201,7 @@
       </c>
       <c r="I23" s="20" t="n">
         <f aca="false">G23/$G$5-1</f>
-        <v>0.0530071355759429</v>
+        <v>0.121606948968513</v>
       </c>
       <c r="J23" s="21" t="n">
         <f aca="false">E23/G23</f>
@@ -5210,7 +5213,7 @@
       </c>
       <c r="L23" s="17" t="n">
         <f aca="false">RANK(H23,$H$5:$H$28)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5240,7 +5243,7 @@
       </c>
       <c r="I24" s="26" t="n">
         <f aca="false">G24/$G$5-1</f>
-        <v>0.0632008154943935</v>
+        <v>0.132464712269273</v>
       </c>
       <c r="J24" s="27" t="n">
         <f aca="false">E24/G24</f>
@@ -5252,7 +5255,7 @@
       </c>
       <c r="L24" s="22" t="n">
         <f aca="false">RANK(H24,$H$5:$H$28)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5282,7 +5285,7 @@
       </c>
       <c r="I25" s="20" t="n">
         <f aca="false">G25/$G$5-1</f>
-        <v>0.142201834862385</v>
+        <v>0.216612377850163</v>
       </c>
       <c r="J25" s="21" t="n">
         <f aca="false">E25/G25</f>
@@ -5324,7 +5327,7 @@
       </c>
       <c r="I26" s="26" t="n">
         <f aca="false">G26/$G$5-1</f>
-        <v>0.632517838939857</v>
+        <v>0.738870792616721</v>
       </c>
       <c r="J26" s="27" t="n">
         <f aca="false">E26/G26</f>
@@ -5332,7 +5335,7 @@
       </c>
       <c r="K26" s="22" t="n">
         <f aca="false">RANK(G26,$G$5:$G$28)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L26" s="22" t="n">
         <f aca="false">RANK(H26,$H$5:$H$28)</f>
@@ -5366,7 +5369,7 @@
       </c>
       <c r="I27" s="33" t="n">
         <f aca="false">G27/$G$5-1</f>
-        <v>0.4072375127421</v>
+        <v>0.498914223669924</v>
       </c>
       <c r="J27" s="34" t="n">
         <f aca="false">E27/G27</f>
@@ -5378,7 +5381,7 @@
       </c>
       <c r="L27" s="29" t="n">
         <f aca="false">RANK(H27,$H$5:$H$28)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5408,7 +5411,7 @@
       </c>
       <c r="I28" s="33" t="n">
         <f aca="false">G28/$G$5-1</f>
-        <v>0.404689092762487</v>
+        <v>0.496199782844734</v>
       </c>
       <c r="J28" s="34" t="n">
         <f aca="false">E28/G28</f>
@@ -5420,7 +5423,7 @@
       </c>
       <c r="L28" s="29" t="n">
         <f aca="false">RANK(H28,$H$5:$H$28)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5512,7 +5515,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
         <v>95</v>
       </c>
@@ -5523,36 +5526,36 @@
         <v>1312</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>882</v>
+        <v>1035</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>970</v>
+        <v>1152</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>1321</v>
+        <v>1327</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>0.9802</v>
+        <v>0.9862</v>
       </c>
       <c r="H5" s="18" t="n">
-        <v>1409</v>
+        <v>1383</v>
       </c>
       <c r="I5" s="18" t="n">
-        <v>1626</v>
+        <v>1586</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>1962</v>
+        <v>1842</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>0.9837</v>
+        <v>0.994</v>
       </c>
       <c r="L5" s="36" t="n">
         <f aca="false">IF(ISNUMBER(C5),F5/C5-1,"n/a")</f>
-        <v>0.00685975609756095</v>
+        <v>0.0114329268292683</v>
       </c>
       <c r="M5" s="20" t="n">
         <f aca="false">J5/F5-1</f>
-        <v>0.485238455715367</v>
+        <v>0.388093443858327</v>
       </c>
       <c r="N5" s="28" t="s">
         <v>177</v>
@@ -5561,7 +5564,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
         <v>97</v>
       </c>
@@ -5572,28 +5575,28 @@
         <v>180</v>
       </c>
       <c r="D6" s="24" t="n">
-        <v>1106</v>
+        <v>734</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>1626</v>
+        <v>1384</v>
       </c>
       <c r="F6" s="24" t="n">
-        <v>1996</v>
+        <v>2259</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>0.9997</v>
+        <v>0.998</v>
       </c>
       <c r="H6" s="24" t="n">
-        <v>323</v>
+        <v>634</v>
       </c>
       <c r="I6" s="24" t="n">
-        <v>570</v>
+        <v>1216</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>1362</v>
+        <v>1883</v>
       </c>
       <c r="K6" s="25" t="n">
-        <v>0.9969</v>
+        <v>0.9968</v>
       </c>
       <c r="L6" s="37" t="str">
         <f aca="false">IF(ISNUMBER(C6),F6/C6-1,"n/a")</f>
@@ -5601,7 +5604,7 @@
       </c>
       <c r="M6" s="26" t="n">
         <f aca="false">J6/F6-1</f>
-        <v>-0.317635270541082</v>
+        <v>-0.166445329791943</v>
       </c>
       <c r="N6" s="23" t="s">
         <v>181</v>
@@ -5621,42 +5624,42 @@
         <v>2192</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>1614</v>
+        <v>1616</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>2036</v>
+        <v>2017</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>2167</v>
+        <v>2186</v>
       </c>
       <c r="G7" s="19" t="n">
-        <v>0.9775</v>
+        <v>0.9886</v>
       </c>
       <c r="H7" s="18" t="n">
         <v>1324</v>
       </c>
       <c r="I7" s="18" t="n">
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>2887</v>
+        <v>3504</v>
       </c>
       <c r="K7" s="19" t="n">
-        <v>0.9867</v>
+        <v>0.9942</v>
       </c>
       <c r="L7" s="36" t="n">
         <f aca="false">IF(ISNUMBER(C7),F7/C7-1,"n/a")</f>
-        <v>-0.011405109489051</v>
+        <v>-0.00273722627737227</v>
       </c>
       <c r="M7" s="20" t="n">
         <f aca="false">J7/F7-1</f>
-        <v>0.332256575911398</v>
+        <v>0.602927721866423</v>
       </c>
       <c r="N7" s="28" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="O7" s="28" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5702,10 +5705,10 @@
         <v>0.81447963800905</v>
       </c>
       <c r="N8" s="22" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O8" s="23" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5751,10 +5754,10 @@
         <v>0.90495867768595</v>
       </c>
       <c r="N9" s="28" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O9" s="28" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5800,15 +5803,15 @@
         <v>0.934455270150576</v>
       </c>
       <c r="N10" s="22" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="O10" s="23" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="35" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -5841,26 +5844,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>92</v>
@@ -5875,16 +5878,16 @@
         <v>24</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5892,7 +5895,7 @@
         <v>137</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>5</v>
@@ -5913,13 +5916,13 @@
         <v>0.9974</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J5" s="20" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K5" s="38" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="L5" s="20" t="n">
         <f aca="false">G5/$G$5-1</f>
@@ -5931,7 +5934,7 @@
         <v>139</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C6" s="22" t="n">
         <v>5</v>
@@ -5973,7 +5976,7 @@
         <v>102</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C7" s="17" t="n">
         <v>5</v>
@@ -6015,7 +6018,7 @@
         <v>141</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C8" s="22" t="n">
         <v>15</v>
@@ -6057,7 +6060,7 @@
         <v>143</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>15</v>
@@ -6099,7 +6102,7 @@
         <v>145</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C10" s="22" t="n">
         <v>5</v>
@@ -6141,7 +6144,7 @@
         <v>147</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>10</v>
@@ -6183,7 +6186,7 @@
         <v>149</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C12" s="22" t="n">
         <v>5</v>
@@ -6225,7 +6228,7 @@
         <v>104</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>5</v>
@@ -6264,10 +6267,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C14" s="22" t="n">
         <v>5</v>
@@ -6306,10 +6309,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="B15" s="17" t="s">
         <v>205</v>
-      </c>
-      <c r="B15" s="17" t="s">
-        <v>204</v>
       </c>
       <c r="C15" s="17" t="n">
         <v>5</v>
@@ -6351,7 +6354,7 @@
         <v>105</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C16" s="22" t="n">
         <v>5</v>
@@ -6393,7 +6396,7 @@
         <v>153</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C17" s="17" t="n">
         <v>10</v>
@@ -6435,7 +6438,7 @@
         <v>155</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C18" s="22" t="n">
         <v>5</v>
@@ -6477,7 +6480,7 @@
         <v>157</v>
       </c>
       <c r="B19" s="29" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C19" s="29" t="n">
         <v>5</v>
@@ -6516,16 +6519,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="29" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B20" s="29" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C20" s="29" t="n">
         <v>5</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E20" s="31" t="n">
         <v>1471</v>
@@ -6561,7 +6564,7 @@
         <v>106</v>
       </c>
       <c r="B21" s="29" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C21" s="29" t="n">
         <v>5</v>
@@ -6600,16 +6603,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="29" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B22" s="29" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C22" s="29" t="n">
         <v>5</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E22" s="31" t="n">
         <v>1716</v>
@@ -6642,17 +6645,17 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="35" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="41" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="42" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B27" s="42" t="s">
         <v>92</v>
@@ -7002,12 +7005,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7015,37 +7018,37 @@
         <v>90</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7091,7 +7094,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B6" s="24" t="n">
         <v>1551</v>
@@ -7132,7 +7135,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>1551</v>
@@ -7173,7 +7176,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B8" s="24" t="n">
         <v>2621</v>
@@ -7214,7 +7217,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B9" s="31" t="n">
         <v>2621</v>
@@ -7283,25 +7286,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>92</v>
@@ -7316,21 +7319,21 @@
         <v>24</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="29" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C6" s="31" t="n">
         <v>2621</v>
@@ -7358,10 +7361,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C7" s="24" t="n">
         <v>2621</v>
@@ -7389,10 +7392,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C8" s="18" t="n">
         <v>2585</v>
@@ -7420,10 +7423,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>2621</v>
@@ -7451,10 +7454,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C10" s="18" t="n">
         <v>1821</v>
@@ -7482,10 +7485,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C11" s="24" t="n">
         <v>2171</v>
@@ -7513,10 +7516,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C12" s="18" t="n">
         <v>1730</v>
@@ -7544,15 +7547,15 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>92</v>
@@ -7567,24 +7570,24 @@
         <v>24</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C17" s="18" t="n">
         <v>2621</v>
@@ -7613,10 +7616,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C18" s="24" t="n">
         <v>2566</v>
@@ -7645,10 +7648,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B19" s="29" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C19" s="31" t="n">
         <v>2621</v>
@@ -7677,10 +7680,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C20" s="24" t="n">
         <v>1471</v>
@@ -7709,10 +7712,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C21" s="18" t="n">
         <v>1696</v>
@@ -7741,10 +7744,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="30" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B22" s="29" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C22" s="31" t="n">
         <v>1716</v>
@@ -7773,7 +7776,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7781,27 +7784,27 @@
         <v>90</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C27" s="18" t="n">
         <v>1688</v>
@@ -7818,10 +7821,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="29" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B28" s="29" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C28" s="31" t="n">
         <v>2618</v>
@@ -7838,10 +7841,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C29" s="18" t="n">
         <v>1152</v>
@@ -7858,10 +7861,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="29" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B30" s="29" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C30" s="31" t="n">
         <v>1487</v>
@@ -7878,7 +7881,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="35" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update thesis files with paper-faithful hybrid results (SH-LEACH, H-LEACH, EECH-HEED) and redraw the family comparison figure
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019rZdtfEbJpAbmcB9G79J6K
</commit_message>
<xml_diff>
--- a/thesis-final/WSN_Protocol_Comparison.xlsx
+++ b/thesis-final/WSN_Protocol_Comparison.xlsx
@@ -352,7 +352,7 @@
     <t xml:space="preserve">Headline</t>
   </si>
   <si>
-    <t xml:space="preserve">v8-Chain FND vs best literature hybrid (H-LEACH Improved)</t>
+    <t xml:space="preserve">v8-Chain FND vs best literature hybrid (SH-LEACH Improved)</t>
   </si>
   <si>
     <t xml:space="preserve">v8-Chain FND vs LEACH</t>
@@ -415,16 +415,16 @@
     <t xml:space="preserve">Literature hybrid</t>
   </si>
   <si>
-    <t xml:space="preserve">LEACH + HEED, single doubling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True iterative doubling, Cprob 0.10→0.03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Energy gate 1.0× average</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Energy gate relaxed to 0.8×</t>
+    <t xml:space="preserve">Eq. 3 literal: round factor keeps growing (≈29 CHs/round)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Round factor made periodic (r mod 1/Cprob)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy gate (&gt; average) + LEACH threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ gate + LEACH G-set (once per 10-round epoch)</t>
   </si>
   <si>
     <t xml:space="preserve">Context</t>
@@ -433,10 +433,10 @@
     <t xml:space="preserve">EECH-HEED</t>
   </si>
   <si>
-    <t xml:space="preserve">HEED + EECH (not LEACH+HEED)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+ adaptive threshold-based sensing (transmits less)</t>
+    <t xml:space="preserve">HEED zone + EECH zone, Eq. 6 threshold, sensing off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zone-2 rotation at the paper's 10 % CH target</t>
   </si>
   <si>
     <t xml:space="preserve">v1</t>
@@ -583,19 +583,19 @@
     <t xml:space="preserve">Lindsey &amp; Raghavendra, 2002 — Table 1 (50×50 m)</t>
   </si>
   <si>
-    <t xml:space="preserve">N = 100, Cprob = 0.10</t>
+    <t xml:space="preserve">N = 100, Cprob = 0.10, Eq. 3 literal (≈29 CHs/round), single-term radio</t>
   </si>
   <si>
     <t xml:space="preserve">Shrestha et al., 2015 — graph only (Fig. 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">With required fallback (literal gate deadlocks)</t>
+    <t xml:space="preserve">Algorithm 1, E_avg over all nodes; fallback needed in 132 rounds</t>
   </si>
   <si>
     <t xml:space="preserve">Razaque et al., 2016 — ≈ read from Fig. 2</t>
   </si>
   <si>
-    <t xml:space="preserve">4000-bit packet</t>
+    <t xml:space="preserve">Paper scenario: 30/70 zones, 56 J, 4000-bit, Eq. 7 sensing on</t>
   </si>
   <si>
     <t xml:space="preserve">Kaur, Kour &amp; Singh, 2025 — Table 7</t>
@@ -1442,10 +1442,10 @@
                   <c:v>1324</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1247</c:v>
+                  <c:v>1480</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2347</c:v>
+                  <c:v>1473</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>1730</c:v>
@@ -1564,10 +1564,10 @@
                   <c:v>2352</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1600</c:v>
+                  <c:v>1542</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2449</c:v>
+                  <c:v>1509</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>2081</c:v>
@@ -1686,10 +1686,10 @@
                   <c:v>3504</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1649</c:v>
+                  <c:v>1558</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2499</c:v>
+                  <c:v>1525</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>2703</c:v>
@@ -1709,11 +1709,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="46280220"/>
-        <c:axId val="52162433"/>
+        <c:axId val="5395512"/>
+        <c:axId val="93571805"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="46280220"/>
+        <c:axId val="5395512"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1745,7 +1745,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52162433"/>
+        <c:crossAx val="93571805"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1753,7 +1753,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52162433"/>
+        <c:axId val="93571805"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1795,7 +1795,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46280220"/>
+        <c:crossAx val="5395512"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1996,10 +1996,10 @@
                   <c:v>0.9942</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.9979</c:v>
+                  <c:v>0.9921</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.9733</c:v>
+                  <c:v>0.9936</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.9772</c:v>
@@ -2019,11 +2019,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="39719945"/>
-        <c:axId val="25492708"/>
+        <c:axId val="90949922"/>
+        <c:axId val="29563077"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="39719945"/>
+        <c:axId val="90949922"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2055,7 +2055,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25492708"/>
+        <c:crossAx val="29563077"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2063,7 +2063,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="25492708"/>
+        <c:axId val="29563077"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2107,7 +2107,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39719945"/>
+        <c:crossAx val="90949922"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2655,11 +2655,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="36069653"/>
-        <c:axId val="94008186"/>
+        <c:axId val="53041961"/>
+        <c:axId val="94741715"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="36069653"/>
+        <c:axId val="53041961"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2691,7 +2691,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94008186"/>
+        <c:crossAx val="94741715"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2699,7 +2699,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94008186"/>
+        <c:axId val="94741715"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2775,7 +2775,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36069653"/>
+        <c:crossAx val="53041961"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3168,11 +3168,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="97603401"/>
-        <c:axId val="69793482"/>
+        <c:axId val="67623910"/>
+        <c:axId val="32179629"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97603401"/>
+        <c:axId val="67623910"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3204,7 +3204,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69793482"/>
+        <c:crossAx val="32179629"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3212,7 +3212,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69793482"/>
+        <c:axId val="32179629"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3288,7 +3288,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97603401"/>
+        <c:crossAx val="67623910"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4164,19 +4164,19 @@
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A8)*('Unified Comparison'!$C$5:$C$28=B8),0),0))</f>
-        <v>1247</v>
+        <v>1480</v>
       </c>
       <c r="D8" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$F$5:$F$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A8)*('Unified Comparison'!$C$5:$C$28=B8),0),0))</f>
-        <v>1600</v>
+        <v>1542</v>
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">INDEX('Unified Comparison'!$G$5:$G$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A8)*('Unified Comparison'!$C$5:$C$28=B8),0),0))</f>
-        <v>1649</v>
+        <v>1558</v>
       </c>
       <c r="F8" s="11" t="n">
         <f aca="false">INDEX('Unified Comparison'!$H$5:$H$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A8)*('Unified Comparison'!$C$5:$C$28=B8),0),0))</f>
-        <v>0.9979</v>
+        <v>0.9921</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4188,19 +4188,19 @@
       </c>
       <c r="C9" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$E$5:$E$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A9)*('Unified Comparison'!$C$5:$C$28=B9),0),0))</f>
-        <v>2347</v>
+        <v>1473</v>
       </c>
       <c r="D9" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$F$5:$F$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A9)*('Unified Comparison'!$C$5:$C$28=B9),0),0))</f>
-        <v>2449</v>
+        <v>1509</v>
       </c>
       <c r="E9" s="8" t="n">
         <f aca="false">INDEX('Unified Comparison'!$G$5:$G$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A9)*('Unified Comparison'!$C$5:$C$28=B9),0),0))</f>
-        <v>2499</v>
+        <v>1525</v>
       </c>
       <c r="F9" s="9" t="n">
         <f aca="false">INDEX('Unified Comparison'!$H$5:$H$28,MATCH(1,INDEX(('Unified Comparison'!$B$5:$B$28=A9)*('Unified Comparison'!$C$5:$C$28=B9),0),0))</f>
-        <v>0.9733</v>
+        <v>0.9936</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4309,8 +4309,8 @@
         <v>108</v>
       </c>
       <c r="C16" s="15" t="n">
-        <f aca="false">C13/C9-1</f>
-        <v>0.116744780570942</v>
+        <f aca="false">C13/C8-1</f>
+        <v>0.770945945945946</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4453,11 +4453,11 @@
       </c>
       <c r="K5" s="17" t="n">
         <f aca="false">RANK(G5,$G$5:$G$28)</f>
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L5" s="17" t="n">
         <f aca="false">RANK(H5,$H$5:$H$28)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="K6" s="22" t="n">
         <f aca="false">RANK(G6,$G$5:$G$28)</f>
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L6" s="22" t="n">
         <f aca="false">RANK(H6,$H$5:$H$28)</f>
@@ -4537,11 +4537,11 @@
       </c>
       <c r="K7" s="17" t="n">
         <f aca="false">RANK(G7,$G$5:$G$28)</f>
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="L7" s="17" t="n">
         <f aca="false">RANK(H7,$H$5:$H$28)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4579,11 +4579,11 @@
       </c>
       <c r="K8" s="22" t="n">
         <f aca="false">RANK(G8,$G$5:$G$28)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" s="22" t="n">
         <f aca="false">RANK(H8,$H$5:$H$28)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4600,32 +4600,32 @@
         <v>129</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>1440</v>
+        <v>647</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>1584</v>
+        <v>702</v>
       </c>
       <c r="G9" s="18" t="n">
-        <v>1604</v>
+        <v>721</v>
       </c>
       <c r="H9" s="19" t="n">
-        <v>0.9917</v>
+        <v>0.9858</v>
       </c>
       <c r="I9" s="20" t="n">
         <f aca="false">G9/$G$5-1</f>
-        <v>-0.129207383279044</v>
+        <v>-0.608577633007601</v>
       </c>
       <c r="J9" s="21" t="n">
         <f aca="false">E9/G9</f>
-        <v>0.897755610972569</v>
+        <v>0.897364771151179</v>
       </c>
       <c r="K9" s="17" t="n">
         <f aca="false">RANK(G9,$G$5:$G$28)</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="L9" s="17" t="n">
         <f aca="false">RANK(H9,$H$5:$H$28)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4642,32 +4642,32 @@
         <v>130</v>
       </c>
       <c r="E10" s="24" t="n">
-        <v>1247</v>
+        <v>1480</v>
       </c>
       <c r="F10" s="24" t="n">
-        <v>1600</v>
+        <v>1542</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>1649</v>
+        <v>1558</v>
       </c>
       <c r="H10" s="25" t="n">
-        <v>0.9979</v>
+        <v>0.9921</v>
       </c>
       <c r="I10" s="26" t="n">
         <f aca="false">G10/$G$5-1</f>
-        <v>-0.104777415852334</v>
+        <v>-0.154180238870793</v>
       </c>
       <c r="J10" s="27" t="n">
         <f aca="false">E10/G10</f>
-        <v>0.756215888417223</v>
+        <v>0.949935815147625</v>
       </c>
       <c r="K10" s="22" t="n">
         <f aca="false">RANK(G10,$G$5:$G$28)</f>
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="L10" s="22" t="n">
         <f aca="false">RANK(H10,$H$5:$H$28)</f>
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4680,36 +4680,36 @@
       <c r="C11" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="28" t="s">
         <v>131</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>2177</v>
+        <v>1384</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>2255</v>
+        <v>1419</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>2305</v>
+        <v>1434</v>
       </c>
       <c r="H11" s="19" t="n">
-        <v>0.9733</v>
+        <v>0.993</v>
       </c>
       <c r="I11" s="20" t="n">
         <f aca="false">G11/$G$5-1</f>
-        <v>0.251357220412595</v>
+        <v>-0.221498371335505</v>
       </c>
       <c r="J11" s="21" t="n">
         <f aca="false">E11/G11</f>
-        <v>0.944468546637744</v>
+        <v>0.96513249651325</v>
       </c>
       <c r="K11" s="17" t="n">
         <f aca="false">RANK(G11,$G$5:$G$28)</f>
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="L11" s="17" t="n">
         <f aca="false">RANK(H11,$H$5:$H$28)</f>
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4722,36 +4722,36 @@
       <c r="C12" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="23" t="s">
         <v>132</v>
       </c>
       <c r="E12" s="24" t="n">
-        <v>2347</v>
+        <v>1473</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>2449</v>
+        <v>1509</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>2499</v>
+        <v>1525</v>
       </c>
       <c r="H12" s="25" t="n">
-        <v>0.9733</v>
+        <v>0.9936</v>
       </c>
       <c r="I12" s="26" t="n">
         <f aca="false">G12/$G$5-1</f>
-        <v>0.356677524429967</v>
+        <v>-0.172095548317047</v>
       </c>
       <c r="J12" s="27" t="n">
         <f aca="false">E12/G12</f>
-        <v>0.939175670268107</v>
+        <v>0.965901639344262</v>
       </c>
       <c r="K12" s="22" t="n">
         <f aca="false">RANK(G12,$G$5:$G$28)</f>
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L12" s="22" t="n">
         <f aca="false">RANK(H12,$H$5:$H$28)</f>
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4764,36 +4764,36 @@
       <c r="C13" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="28" t="s">
         <v>135</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>1653</v>
+        <v>1311</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>2134</v>
+        <v>1382</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>2184</v>
+        <v>1545</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>0.9168</v>
+        <v>0.9974</v>
       </c>
       <c r="I13" s="20" t="n">
         <f aca="false">G13/$G$5-1</f>
-        <v>0.185667752442997</v>
+        <v>-0.161237785016287</v>
       </c>
       <c r="J13" s="21" t="n">
         <f aca="false">E13/G13</f>
-        <v>0.756868131868132</v>
+        <v>0.848543689320388</v>
       </c>
       <c r="K13" s="17" t="n">
         <f aca="false">RANK(G13,$G$5:$G$28)</f>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="L13" s="17" t="n">
         <f aca="false">RANK(H13,$H$5:$H$28)</f>
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4810,32 +4810,32 @@
         <v>136</v>
       </c>
       <c r="E14" s="24" t="n">
-        <v>2502</v>
+        <v>1368</v>
       </c>
       <c r="F14" s="24" t="n">
-        <v>3758</v>
+        <v>1385</v>
       </c>
       <c r="G14" s="24" t="n">
-        <v>3808</v>
+        <v>1767</v>
       </c>
       <c r="H14" s="25" t="n">
-        <v>0.9214</v>
+        <v>0.9951</v>
       </c>
       <c r="I14" s="26" t="n">
         <f aca="false">G14/$G$5-1</f>
-        <v>1.06731813246471</v>
+        <v>-0.0407166123778502</v>
       </c>
       <c r="J14" s="27" t="n">
         <f aca="false">E14/G14</f>
-        <v>0.65703781512605</v>
+        <v>0.774193548387097</v>
       </c>
       <c r="K14" s="22" t="n">
         <f aca="false">RANK(G14,$G$5:$G$28)</f>
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="L14" s="22" t="n">
         <f aca="false">RANK(H14,$H$5:$H$28)</f>
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4873,11 +4873,11 @@
       </c>
       <c r="K15" s="17" t="n">
         <f aca="false">RANK(G15,$G$5:$G$28)</f>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L15" s="17" t="n">
         <f aca="false">RANK(H15,$H$5:$H$28)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="K16" s="22" t="n">
         <f aca="false">RANK(G16,$G$5:$G$28)</f>
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L16" s="22" t="n">
         <f aca="false">RANK(H16,$H$5:$H$28)</f>
@@ -4957,11 +4957,11 @@
       </c>
       <c r="K17" s="17" t="n">
         <f aca="false">RANK(G17,$G$5:$G$28)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L17" s="17" t="n">
         <f aca="false">RANK(H17,$H$5:$H$28)</f>
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4999,11 +4999,11 @@
       </c>
       <c r="K18" s="22" t="n">
         <f aca="false">RANK(G18,$G$5:$G$28)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L18" s="22" t="n">
         <f aca="false">RANK(H18,$H$5:$H$28)</f>
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5041,11 +5041,11 @@
       </c>
       <c r="K19" s="17" t="n">
         <f aca="false">RANK(G19,$G$5:$G$28)</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L19" s="17" t="n">
         <f aca="false">RANK(H19,$H$5:$H$28)</f>
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="K20" s="22" t="n">
         <f aca="false">RANK(G20,$G$5:$G$28)</f>
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="L20" s="22" t="n">
         <f aca="false">RANK(H20,$H$5:$H$28)</f>
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5125,11 +5125,11 @@
       </c>
       <c r="K21" s="17" t="n">
         <f aca="false">RANK(G21,$G$5:$G$28)</f>
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="L21" s="17" t="n">
         <f aca="false">RANK(H21,$H$5:$H$28)</f>
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5167,11 +5167,11 @@
       </c>
       <c r="K22" s="22" t="n">
         <f aca="false">RANK(G22,$G$5:$G$28)</f>
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="L22" s="22" t="n">
         <f aca="false">RANK(H22,$H$5:$H$28)</f>
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5209,11 +5209,11 @@
       </c>
       <c r="K23" s="17" t="n">
         <f aca="false">RANK(G23,$G$5:$G$28)</f>
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L23" s="17" t="n">
         <f aca="false">RANK(H23,$H$5:$H$28)</f>
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5251,11 +5251,11 @@
       </c>
       <c r="K24" s="22" t="n">
         <f aca="false">RANK(G24,$G$5:$G$28)</f>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="L24" s="22" t="n">
         <f aca="false">RANK(H24,$H$5:$H$28)</f>
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5293,11 +5293,11 @@
       </c>
       <c r="K25" s="17" t="n">
         <f aca="false">RANK(G25,$G$5:$G$28)</f>
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="L25" s="17" t="n">
         <f aca="false">RANK(H25,$H$5:$H$28)</f>
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5335,11 +5335,11 @@
       </c>
       <c r="K26" s="22" t="n">
         <f aca="false">RANK(G26,$G$5:$G$28)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L26" s="22" t="n">
         <f aca="false">RANK(H26,$H$5:$H$28)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5377,11 +5377,11 @@
       </c>
       <c r="K27" s="29" t="n">
         <f aca="false">RANK(G27,$G$5:$G$28)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L27" s="29" t="n">
         <f aca="false">RANK(H27,$H$5:$H$28)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5419,11 +5419,11 @@
       </c>
       <c r="K28" s="29" t="n">
         <f aca="false">RANK(G28,$G$5:$G$28)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L28" s="29" t="n">
         <f aca="false">RANK(H28,$H$5:$H$28)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5662,7 +5662,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
         <v>99</v>
       </c>
@@ -5673,28 +5673,28 @@
         <v>180</v>
       </c>
       <c r="D8" s="24" t="n">
-        <v>493</v>
+        <v>484</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>747</v>
+        <v>583</v>
       </c>
       <c r="F8" s="24" t="n">
-        <v>884</v>
+        <v>689</v>
       </c>
       <c r="G8" s="25" t="n">
-        <v>0.9953</v>
+        <v>0.9966</v>
       </c>
       <c r="H8" s="24" t="n">
-        <v>1440</v>
+        <v>647</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>1584</v>
+        <v>702</v>
       </c>
       <c r="J8" s="24" t="n">
-        <v>1604</v>
+        <v>721</v>
       </c>
       <c r="K8" s="25" t="n">
-        <v>0.9917</v>
+        <v>0.9858</v>
       </c>
       <c r="L8" s="37" t="str">
         <f aca="false">IF(ISNUMBER(C8),F8/C8-1,"n/a")</f>
@@ -5702,16 +5702,16 @@
       </c>
       <c r="M8" s="26" t="n">
         <f aca="false">J8/F8-1</f>
-        <v>0.81447963800905</v>
-      </c>
-      <c r="N8" s="22" t="s">
+        <v>0.04644412191582</v>
+      </c>
+      <c r="N8" s="23" t="s">
         <v>185</v>
       </c>
       <c r="O8" s="23" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
         <v>101</v>
       </c>
@@ -5722,36 +5722,36 @@
         <v>4312</v>
       </c>
       <c r="D9" s="18" t="n">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>1160</v>
+        <v>1157</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>1210</v>
+        <v>1207</v>
       </c>
       <c r="G9" s="19" t="n">
-        <v>0.9475</v>
+        <v>0.9504</v>
       </c>
       <c r="H9" s="18" t="n">
-        <v>2177</v>
+        <v>1384</v>
       </c>
       <c r="I9" s="18" t="n">
-        <v>2255</v>
+        <v>1419</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>2305</v>
+        <v>1434</v>
       </c>
       <c r="K9" s="19" t="n">
-        <v>0.9733</v>
+        <v>0.993</v>
       </c>
       <c r="L9" s="36" t="n">
         <f aca="false">IF(ISNUMBER(C9),F9/C9-1,"n/a")</f>
-        <v>-0.719387755102041</v>
+        <v>-0.720083487940631</v>
       </c>
       <c r="M9" s="20" t="n">
         <f aca="false">J9/F9-1</f>
-        <v>0.90495867768595</v>
+        <v>0.188069594034797</v>
       </c>
       <c r="N9" s="28" t="s">
         <v>187</v>
@@ -5760,7 +5760,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
         <v>134</v>
       </c>
@@ -5771,38 +5771,38 @@
         <v>2200</v>
       </c>
       <c r="D10" s="24" t="n">
-        <v>792</v>
+        <v>1121</v>
       </c>
       <c r="E10" s="24" t="n">
-        <v>1079</v>
+        <v>1954</v>
       </c>
       <c r="F10" s="24" t="n">
-        <v>1129</v>
+        <v>3783</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>0.9043</v>
+        <v>0.9978</v>
       </c>
       <c r="H10" s="24" t="n">
-        <v>1653</v>
+        <v>1311</v>
       </c>
       <c r="I10" s="24" t="n">
-        <v>2134</v>
+        <v>1382</v>
       </c>
       <c r="J10" s="24" t="n">
-        <v>2184</v>
+        <v>1545</v>
       </c>
       <c r="K10" s="25" t="n">
-        <v>0.9168</v>
+        <v>0.9974</v>
       </c>
       <c r="L10" s="37" t="n">
         <f aca="false">IF(ISNUMBER(C10),F10/C10-1,"n/a")</f>
-        <v>-0.486818181818182</v>
+        <v>0.719545454545455</v>
       </c>
       <c r="M10" s="26" t="n">
         <f aca="false">J10/F10-1</f>
-        <v>0.934455270150576</v>
-      </c>
-      <c r="N10" s="22" t="s">
+        <v>-0.591593973037272</v>
+      </c>
+      <c r="N10" s="23" t="s">
         <v>189</v>
       </c>
       <c r="O10" s="23" t="s">

</xml_diff>